<commit_message>
Business: board, small parts and JLCPCB assembly priced from published LCSC/JLCPCB rates; device without enclosure ~ $16.8
</commit_message>
<xml_diff>
--- a/business/afib_unit_economics.xlsx
+++ b/business/afib_unit_economics.xlsx
@@ -9,9 +9,10 @@
   </bookViews>
   <sheets>
     <sheet name="Допущения" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Юнит-экономика" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Сравнение" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Чего не хватает" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Плата и сборка" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Юнит-экономика" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Сравнение" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Чего не хватает" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="208">
   <si>
     <t xml:space="preserve">AFib Monitor — допущения для цены и юнит-экономики</t>
   </si>
@@ -79,10 +80,10 @@
     <t xml:space="preserve">Adafruit #1317, розница за 1 шт: $5.95 — верхняя граница, оптом дешевле</t>
   </si>
   <si>
-    <t xml:space="preserve">Плата, пассивные элементы, сборка, корпус, упаковка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">НЕТ ДАННЫХ — нужна котировка производителя плат (например JLCPCB/PCBWay) по нашей схеме. Пока пусто = себестоимость ниже реальной.</t>
+    <t xml:space="preserve">Остальные детали платы, сама плата и сборка (лист «Плата и сборка»)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Считается на листе «Плата и сборка» по ценам LCSC и тарифам JLCPCB. Корпус и кабель к электродам НЕ включены — нет данных.</t>
   </si>
   <si>
     <t xml:space="preserve">Расходники</t>
@@ -241,25 +242,202 @@
     <t xml:space="preserve">«AF is estimated to affect 2-4% of the adult population worldwide» — Lancet Reg Health West Pac 2022 (PMC9252928), со ссылкой на ESC 2020. Для КР своих данных не нашёл.</t>
   </si>
   <si>
+    <t xml:space="preserve">Плата и сборка: детали (LCSC) и сборка (JLCPCB, Economic PCBA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Цены деталей — за 1 шт при ~100 шт (если нет тарифа 100+ — ближайший). Пайки — по числу выводов корпуса, ОЦЕНКА: проверить по футпринтам. Главные детали (ESP32, AD8232, аккумулятор) — на листе «Допущения».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Деталь</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Номер LCSC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кол-во</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Цена, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Паек на шт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сумма, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Зарядка LiPo MCP73831T-2ACI/OT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C424093</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C424093.html, 100+: $0.4483</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Стабилизатор 3.3 В ME6211C33M5G-N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C82942</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C82942.html, 100+: $0.0503</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Разъём USB-C TYPE-C-31-M-12 (16 конт.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C165948</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C165948.html, 50+: $0.1368 (тарифа 100+ нет)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Гнездо 3.5 мм для кабеля электродов KH-PJ-321A-SMT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5123133</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C5123133.html, 50+: $0.0819 (большая из двух цен)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Разъём аккумулятора JST B2B-PH-K-S (выводной)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C131337</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C131337.html, 20+: $0.0358; паяется вручную</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Резисторы 0402 (обвязка AD8232, делитель батареи, светодиод)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C25744</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C25744.html, 100+: $0.0016. Количество — ОЦЕНКА по типовой схеме AD8232</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Конденсаторы 0402 100 нФ и др.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1525</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C1525.html, 100+: $0.004. Количество — ОЦЕНКА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP32-S3-MINI-1 и AD8232 (пайки; цены — на листе «Допущения»)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ОЦЕНКА: 65 площадок модуля + 21 у AD8232 (LFCSP-20 + теплоотвод); проверить по футпринтам</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Цена 5 плат 2 слоя до 100×100 мм (акция)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/pcba/price: «1-2 layer, 100x100mm … the pcb cost is $2»; для партии 100 шт уточнить калькулятором</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Плат в партии</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Меняйте</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Типов «Extended»-деталей (за каждый — загрузка питателя)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Допущение: ESP32, AD8232, MCP73831, USB-C, гнездо 3.5 мм, ME6211 — все Extended</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMT-пайка, $ за пайку (Economic)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jlcpcb.com/help/article/pcb-assembly-price: 1–100 000 паек</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ручная сборка, $ за пайку</t>
+  </si>
+  <si>
+    <t xml:space="preserve">там же: 1–10 000 паек</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Наладка (Economic), за заказ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">там же</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Трафарет (Economic), за заказ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Загрузка питателя за Extended-деталь</t>
+  </si>
+  <si>
+    <t xml:space="preserve">там же: «$3.07 for Extended»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ручная пайка, за заказ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">там же: «Hand-soldering labor $3.58 per order»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Мелкие детали на плату</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Паек SMT на плату</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Без выводного разъёма аккумулятора</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMT-пайка на плату</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ручная пайка разъёма на плату</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сама плата, за 1 шт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Постоянные расходы на партию</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Наладка + трафарет + питатели + ручная пайка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Постоянные расходы на 1 плату</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ИТОГО на одну плату (без ESP32, AD8232, аккумулятора, корпуса)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Идёт в «Допущения» → себестоимость устройства</t>
+  </si>
+  <si>
     <t xml:space="preserve">Юнит-экономика (все суммы в сомах, без НДС и таможни)</t>
   </si>
   <si>
     <t xml:space="preserve">Устройство</t>
   </si>
   <si>
-    <t xml:space="preserve">Себестоимость известных деталей, $</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Без платы, сборки и корпуса, пока их нет в «Допущениях»</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Себестоимость известных деталей, сом</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Валовая маржа на устройстве (по известным деталям)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Завышена, пока не добавлены плата, сборка, корпус</t>
+    <t xml:space="preserve">Себестоимость платы с деталями и сборкой, $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Без корпуса и кабеля к электродам</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Себестоимость платы с деталями и сборкой, сом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Валовая маржа на устройстве (без корпуса)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Завышена на стоимость корпуса, кабеля, упаковки, доставки и пошлин</t>
   </si>
   <si>
     <t xml:space="preserve">Маржа, % от цены</t>
@@ -409,13 +587,13 @@
     <t xml:space="preserve">Кто</t>
   </si>
   <si>
-    <t xml:space="preserve">Котировка на плату, сборку, корпус</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сейчас в себестоимости только 3 детали; без этого маржа завышена</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Я: схема → запрос JLCPCB/PCBWay</t>
+    <t xml:space="preserve">Корпус и кабель к электродам; точная цена платы для 100 шт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Плата и сборка посчитаны по тарифам, но корпус не посчитан; цена самой платы взята как акция $2 за 5 шт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Я: схема в KiCad → калькулятор JLCPCB; корпус — 3D-печать или литьё</t>
   </si>
   <si>
     <t xml:space="preserve">Регистрация медизделия в ЕАЭС / КР: класс, сроки, стоимость испытаний</t>
@@ -476,14 +654,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="167" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="168" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="169" formatCode="#,##0&quot; сом&quot;;\(#,##0&quot; сом)&quot;;\-"/>
-    <numFmt numFmtId="170" formatCode="0.0\x"/>
+    <numFmt numFmtId="170" formatCode="\$0.0000"/>
+    <numFmt numFmtId="171" formatCode="\$0.00"/>
+    <numFmt numFmtId="172" formatCode="0"/>
+    <numFmt numFmtId="173" formatCode="\$0.000"/>
+    <numFmt numFmtId="174" formatCode="0.0\x"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -604,7 +786,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -645,7 +827,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -673,6 +855,46 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -689,7 +911,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1079,7 +1301,10 @@
       <c r="A10" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="10"/>
+      <c r="B10" s="10" t="n">
+        <f aca="false">'Плата и сборка'!$B$31</f>
+        <v>1.855</v>
+      </c>
       <c r="C10" s="7" t="s">
         <v>12</v>
       </c>
@@ -1412,12 +1637,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1425,314 +1654,411 @@
         <v>72</v>
       </c>
     </row>
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>73</v>
+      <c r="A3" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B4" s="17" t="n">
-        <f aca="false">Допущения!$B$7+Допущения!$B$8+Допущения!$B$9+Допущения!$B$10</f>
-        <v>14.9728</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>75</v>
+      <c r="A4" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="18" t="n">
+        <v>0.4483</v>
+      </c>
+      <c r="E4" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <f aca="false">C4*D4</f>
+        <v>0.4483</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B5" s="18" t="n">
-        <f aca="false">B4*Допущения!$B$5</f>
-        <v>1309.37136</v>
-      </c>
-      <c r="E5" s="7"/>
+      <c r="A5" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="18" t="n">
+        <v>0.0503</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <f aca="false">C5*D5</f>
+        <v>0.0503</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B6" s="18" t="n">
-        <f aca="false">Допущения!$B$22</f>
-        <v>6900</v>
-      </c>
-      <c r="E6" s="7"/>
+      <c r="A6" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>0.1368</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <f aca="false">C6*D6</f>
+        <v>0.1368</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B7" s="18" t="n">
-        <f aca="false">B6-B5</f>
-        <v>5590.62864</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>78</v>
+      <c r="A7" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>0.0819</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <f aca="false">C7*D7</f>
+        <v>0.0819</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B8" s="19" t="n">
-        <f aca="false">IF(B6=0,0,B7/B6)</f>
-        <v>0.810236034782609</v>
-      </c>
-      <c r="E8" s="7"/>
+      <c r="A8" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>0.0358</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <f aca="false">C8*D8</f>
+        <v>0.0358</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <f aca="false">C9*D9</f>
+        <v>0.0192</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>80</v>
+      <c r="A10" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <f aca="false">C10*D10</f>
+        <v>0.056</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="B11" s="11" t="n">
-        <v>50</v>
-      </c>
-      <c r="C11" s="11" t="n">
-        <v>200</v>
-      </c>
-      <c r="D11" s="11" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B12" s="18" t="n">
-        <f aca="false">Допущения!$B$23</f>
-        <v>390</v>
-      </c>
-      <c r="C12" s="18" t="n">
-        <f aca="false">Допущения!$B$23</f>
-        <v>390</v>
-      </c>
-      <c r="D12" s="18" t="n">
-        <f aca="false">Допущения!$B$23</f>
-        <v>390</v>
-      </c>
-      <c r="E12" s="7"/>
+      <c r="A11" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="B13" s="18" t="n">
-        <f aca="false">Допущения!$B$23*Допущения!$B$19*Допущения!$B$20</f>
-        <v>58.5</v>
-      </c>
-      <c r="C13" s="18" t="n">
-        <f aca="false">Допущения!$B$23*Допущения!$B$19*Допущения!$B$20</f>
-        <v>58.5</v>
-      </c>
-      <c r="D13" s="18" t="n">
-        <f aca="false">Допущения!$B$23*Допущения!$B$19*Допущения!$B$20</f>
-        <v>58.5</v>
-      </c>
-      <c r="E13" s="7"/>
+      <c r="A13" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B14" s="18" t="n">
-        <f aca="false">(Допущения!$B$15+Допущения!$B$16)*Допущения!$B$5/B11</f>
-        <v>22.737</v>
-      </c>
-      <c r="C14" s="18" t="n">
-        <f aca="false">(Допущения!$B$15+Допущения!$B$16)*Допущения!$B$5/C11</f>
-        <v>5.68425</v>
-      </c>
-      <c r="D14" s="18" t="n">
-        <f aca="false">(Допущения!$B$15+Допущения!$B$16)*Допущения!$B$5/D11</f>
-        <v>1.13685</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>86</v>
+      <c r="A14" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="B14" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="B15" s="18" t="n">
-        <f aca="false">(Допущения!$B$17/12)*Допущения!$B$5/B11</f>
-        <v>14.42925</v>
-      </c>
-      <c r="C15" s="18" t="n">
-        <f aca="false">(Допущения!$B$17/12)*Допущения!$B$5/C11</f>
-        <v>3.6073125</v>
-      </c>
-      <c r="D15" s="18" t="n">
-        <f aca="false">(Допущения!$B$17/12)*Допущения!$B$5/D11</f>
-        <v>0.7214625</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>88</v>
+      <c r="A15" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B16" s="20" t="n">
-        <f aca="false">B12-B13-B14-B15</f>
-        <v>294.33375</v>
-      </c>
-      <c r="C16" s="20" t="n">
-        <f aca="false">C12-C13-C14-C15</f>
-        <v>322.2084375</v>
-      </c>
-      <c r="D16" s="20" t="n">
-        <f aca="false">D12-D13-D14-D15</f>
-        <v>329.6416875</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>90</v>
+      <c r="A16" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" s="18" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
-        <v>91</v>
+      <c r="A17" s="0" t="s">
+        <v>111</v>
       </c>
       <c r="B17" s="18" t="n">
-        <f aca="false">B16*B11</f>
-        <v>14716.6875</v>
-      </c>
-      <c r="C17" s="18" t="n">
-        <f aca="false">C16*C11</f>
-        <v>64441.6875</v>
-      </c>
-      <c r="D17" s="18" t="n">
-        <f aca="false">D16*D11</f>
-        <v>329641.6875</v>
-      </c>
-      <c r="E17" s="7"/>
+        <v>0.0164</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="B18" s="20" t="n">
-        <f aca="false">B17*12</f>
-        <v>176600.25</v>
-      </c>
-      <c r="C18" s="20" t="n">
-        <f aca="false">C17*12</f>
-        <v>773300.25</v>
-      </c>
-      <c r="D18" s="20" t="n">
-        <f aca="false">D17*12</f>
-        <v>3955700.25</v>
-      </c>
-      <c r="E18" s="7"/>
+      <c r="A18" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="B18" s="22" t="n">
+        <v>8.18</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="B19" s="22" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
-        <v>93</v>
+      <c r="A20" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="B20" s="22" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B21" s="18" t="n">
-        <f aca="false">Допущения!$B$12*Допущения!$B$13*Допущения!$B$5</f>
-        <v>865.755</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B22" s="18" t="n">
-        <f aca="false">B21*(1+Допущения!$B$24)</f>
-        <v>1038.906</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>97</v>
+      <c r="A21" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="B21" s="22" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="B23" s="21" t="n">
-        <f aca="false">IF(Допущения!$B$23=0,0,B21/Допущения!$B$23)</f>
-        <v>2.21988461538462</v>
-      </c>
-      <c r="E23" s="7"/>
+      <c r="A23" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="B23" s="23" t="n">
+        <f aca="false">SUM(F4:F10)</f>
+        <v>0.8283</v>
+      </c>
+      <c r="G23" s="7"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="B24" s="18" t="n">
-        <f aca="false">Допущения!$B$23+B22</f>
-        <v>1428.906</v>
-      </c>
-      <c r="E24" s="7"/>
+      <c r="A24" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="B24" s="24" t="n">
+        <f aca="false">SUMPRODUCT(C4:C11,E4:E11)-C8*E8</f>
+        <v>173</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="B25" s="19" t="n">
-        <f aca="false">IF(Допущения!$B$32=0,0,B24/Допущения!$B$32)</f>
-        <v>0.0275382747456059</v>
-      </c>
-      <c r="E25" s="7"/>
+      <c r="A25" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="B25" s="23" t="n">
+        <f aca="false">B24*B16</f>
+        <v>0.2768</v>
+      </c>
+      <c r="G25" s="7"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="B26" s="23" t="n">
+        <f aca="false">C8*E8*B17</f>
+        <v>0.0328</v>
+      </c>
+      <c r="G26" s="7"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
-        <v>101</v>
-      </c>
+      <c r="A27" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="B27" s="23" t="n">
+        <f aca="false">B13/5</f>
+        <v>0.4</v>
+      </c>
+      <c r="G27" s="7"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="B28" s="22" t="n">
-        <f aca="false">(Допущения!$B$15+Допущения!$B$16+Допущения!$B$17/12)*Допущения!$B$5</f>
-        <v>1858.3125</v>
+      <c r="A28" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="B28" s="25" t="n">
+        <f aca="false">B18+B19+B15*B20+B21</f>
+        <v>31.71</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="B29" s="22" t="n">
-        <f aca="false">Допущения!$B$23*(1-Допущения!$B$19*Допущения!$B$20)</f>
-        <v>331.5</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="B30" s="23" t="n">
-        <f aca="false">IF(B29&lt;=0,0,ROUNDUP(B28/B29,0))</f>
-        <v>6</v>
-      </c>
-      <c r="E30" s="7" t="s">
-        <v>105</v>
+      <c r="A29" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="B29" s="23" t="n">
+        <f aca="false">IF(B14=0,0,B28/B14)</f>
+        <v>0.3171</v>
+      </c>
+      <c r="G29" s="7"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B31" s="26" t="n">
+        <f aca="false">B23+B25+B26+B27+B29</f>
+        <v>1.855</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1748,137 +2074,324 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>110</v>
+      <c r="A3" s="4" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
-        <v>111</v>
-      </c>
-      <c r="B4" s="25" t="n">
-        <f aca="false">Допущения!$B$22+12*'Юнит-экономика'!B24</f>
-        <v>24046.872</v>
-      </c>
-      <c r="C4" s="26" t="n">
-        <f aca="false">IF(Допущения!$B$32=0,0,B4/(12*Допущения!$B$32))</f>
-        <v>0.0386198350292939</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
-        <v>113</v>
-      </c>
-      <c r="B5" s="18" t="n">
-        <f aca="false">Допущения!$B$22+12*Допущения!$B$23</f>
-        <v>11580</v>
-      </c>
-      <c r="C5" s="26" t="n">
-        <f aca="false">IF(Допущения!$B$32=0,0,B5/(12*Допущения!$B$32))</f>
-        <v>0.0185977489978415</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>114</v>
-      </c>
+      <c r="A4" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" s="27" t="n">
+        <f aca="false">Допущения!$B$7+Допущения!$B$8+Допущения!$B$9+Допущения!$B$10</f>
+        <v>16.8278</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B5" s="28" t="n">
+        <f aca="false">B4*Допущения!$B$5</f>
+        <v>1471.59111</v>
+      </c>
+      <c r="E5" s="7"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
-        <v>115</v>
-      </c>
-      <c r="B6" s="18" t="n">
-        <f aca="false">4*Допущения!$B$26</f>
-        <v>6000</v>
-      </c>
-      <c r="C6" s="26" t="n">
-        <f aca="false">IF(Допущения!$B$32=0,0,B6/(12*Допущения!$B$32))</f>
-        <v>0.00963613937711995</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>116</v>
-      </c>
+      <c r="A6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="28" t="n">
+        <f aca="false">Допущения!$B$22</f>
+        <v>6900</v>
+      </c>
+      <c r="E6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
-        <v>117</v>
-      </c>
-      <c r="B7" s="18" t="n">
-        <f aca="false">4*Допущения!$B$27</f>
-        <v>7200</v>
-      </c>
-      <c r="C7" s="26" t="n">
-        <f aca="false">IF(Допущения!$B$32=0,0,B7/(12*Допущения!$B$32))</f>
-        <v>0.0115633672525439</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="24" t="s">
-        <v>118</v>
-      </c>
-      <c r="B8" s="18" t="n">
-        <f aca="false">(Допущения!$B$30+Допущения!$B$31)*Допущения!$B$5</f>
-        <v>30432.6</v>
-      </c>
-      <c r="C8" s="26" t="n">
-        <f aca="false">IF(Допущения!$B$32=0,0,B8/(12*Допущения!$B$32))</f>
-        <v>0.0488754625346901</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>119</v>
+      <c r="A7" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B7" s="28" t="n">
+        <f aca="false">B6-B5</f>
+        <v>5428.40889</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="B8" s="29" t="n">
+        <f aca="false">IF(B6=0,0,B7/B6)</f>
+        <v>0.786725926086957</v>
+      </c>
+      <c r="E8" s="7"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
-        <v>121</v>
-      </c>
-      <c r="B12" s="27" t="n">
-        <f aca="false">Допущения!$B$34*Допущения!$B$35</f>
-        <v>9500</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24" t="s">
-        <v>123</v>
+        <v>140</v>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>200</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B12" s="28" t="n">
+        <f aca="false">Допущения!$B$23</f>
+        <v>390</v>
+      </c>
+      <c r="C12" s="28" t="n">
+        <f aca="false">Допущения!$B$23</f>
+        <v>390</v>
+      </c>
+      <c r="D12" s="28" t="n">
+        <f aca="false">Допущения!$B$23</f>
+        <v>390</v>
+      </c>
+      <c r="E12" s="7"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>143</v>
       </c>
       <c r="B13" s="28" t="n">
-        <f aca="false">'Юнит-экономика'!B30</f>
+        <f aca="false">Допущения!$B$23*Допущения!$B$19*Допущения!$B$20</f>
+        <v>58.5</v>
+      </c>
+      <c r="C13" s="28" t="n">
+        <f aca="false">Допущения!$B$23*Допущения!$B$19*Допущения!$B$20</f>
+        <v>58.5</v>
+      </c>
+      <c r="D13" s="28" t="n">
+        <f aca="false">Допущения!$B$23*Допущения!$B$19*Допущения!$B$20</f>
+        <v>58.5</v>
+      </c>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="B14" s="28" t="n">
+        <f aca="false">(Допущения!$B$15+Допущения!$B$16)*Допущения!$B$5/B11</f>
+        <v>22.737</v>
+      </c>
+      <c r="C14" s="28" t="n">
+        <f aca="false">(Допущения!$B$15+Допущения!$B$16)*Допущения!$B$5/C11</f>
+        <v>5.68425</v>
+      </c>
+      <c r="D14" s="28" t="n">
+        <f aca="false">(Допущения!$B$15+Допущения!$B$16)*Допущения!$B$5/D11</f>
+        <v>1.13685</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="B15" s="28" t="n">
+        <f aca="false">(Допущения!$B$17/12)*Допущения!$B$5/B11</f>
+        <v>14.42925</v>
+      </c>
+      <c r="C15" s="28" t="n">
+        <f aca="false">(Допущения!$B$17/12)*Допущения!$B$5/C11</f>
+        <v>3.6073125</v>
+      </c>
+      <c r="D15" s="28" t="n">
+        <f aca="false">(Допущения!$B$17/12)*Допущения!$B$5/D11</f>
+        <v>0.7214625</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B16" s="30" t="n">
+        <f aca="false">B12-B13-B14-B15</f>
+        <v>294.33375</v>
+      </c>
+      <c r="C16" s="30" t="n">
+        <f aca="false">C12-C13-C14-C15</f>
+        <v>322.2084375</v>
+      </c>
+      <c r="D16" s="30" t="n">
+        <f aca="false">D12-D13-D14-D15</f>
+        <v>329.6416875</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B17" s="28" t="n">
+        <f aca="false">B16*B11</f>
+        <v>14716.6875</v>
+      </c>
+      <c r="C17" s="28" t="n">
+        <f aca="false">C16*C11</f>
+        <v>64441.6875</v>
+      </c>
+      <c r="D17" s="28" t="n">
+        <f aca="false">D16*D11</f>
+        <v>329641.6875</v>
+      </c>
+      <c r="E17" s="7"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B18" s="30" t="n">
+        <f aca="false">B17*12</f>
+        <v>176600.25</v>
+      </c>
+      <c r="C18" s="30" t="n">
+        <f aca="false">C17*12</f>
+        <v>773300.25</v>
+      </c>
+      <c r="D18" s="30" t="n">
+        <f aca="false">D17*12</f>
+        <v>3955700.25</v>
+      </c>
+      <c r="E18" s="7"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="B21" s="28" t="n">
+        <f aca="false">Допущения!$B$12*Допущения!$B$13*Допущения!$B$5</f>
+        <v>865.755</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B22" s="28" t="n">
+        <f aca="false">B21*(1+Допущения!$B$24)</f>
+        <v>1038.906</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B23" s="31" t="n">
+        <f aca="false">IF(Допущения!$B$23=0,0,B21/Допущения!$B$23)</f>
+        <v>2.21988461538462</v>
+      </c>
+      <c r="E23" s="7"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="B24" s="28" t="n">
+        <f aca="false">Допущения!$B$23+B22</f>
+        <v>1428.906</v>
+      </c>
+      <c r="E24" s="7"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="B25" s="29" t="n">
+        <f aca="false">IF(Допущения!$B$32=0,0,B24/Допущения!$B$32)</f>
+        <v>0.0275382747456059</v>
+      </c>
+      <c r="E25" s="7"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="B28" s="32" t="n">
+        <f aca="false">(Допущения!$B$15+Допущения!$B$16+Допущения!$B$17/12)*Допущения!$B$5</f>
+        <v>1858.3125</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="B29" s="32" t="n">
+        <f aca="false">Допущения!$B$23*(1-Допущения!$B$19*Допущения!$B$20)</f>
+        <v>331.5</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="B30" s="33" t="n">
+        <f aca="false">IF(B29&lt;=0,0,ROUNDUP(B28/B29,0))</f>
         <v>6</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -1897,6 +2410,155 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="34" t="s">
+        <v>170</v>
+      </c>
+      <c r="B4" s="35" t="n">
+        <f aca="false">Допущения!$B$22+12*'Юнит-экономика'!B24</f>
+        <v>24046.872</v>
+      </c>
+      <c r="C4" s="36" t="n">
+        <f aca="false">IF(Допущения!$B$32=0,0,B4/(12*Допущения!$B$32))</f>
+        <v>0.0386198350292939</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="34" t="s">
+        <v>172</v>
+      </c>
+      <c r="B5" s="28" t="n">
+        <f aca="false">Допущения!$B$22+12*Допущения!$B$23</f>
+        <v>11580</v>
+      </c>
+      <c r="C5" s="36" t="n">
+        <f aca="false">IF(Допущения!$B$32=0,0,B5/(12*Допущения!$B$32))</f>
+        <v>0.0185977489978415</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="34" t="s">
+        <v>174</v>
+      </c>
+      <c r="B6" s="28" t="n">
+        <f aca="false">4*Допущения!$B$26</f>
+        <v>6000</v>
+      </c>
+      <c r="C6" s="36" t="n">
+        <f aca="false">IF(Допущения!$B$32=0,0,B6/(12*Допущения!$B$32))</f>
+        <v>0.00963613937711995</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="34" t="s">
+        <v>176</v>
+      </c>
+      <c r="B7" s="28" t="n">
+        <f aca="false">4*Допущения!$B$27</f>
+        <v>7200</v>
+      </c>
+      <c r="C7" s="36" t="n">
+        <f aca="false">IF(Допущения!$B$32=0,0,B7/(12*Допущения!$B$32))</f>
+        <v>0.0115633672525439</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="34" t="s">
+        <v>177</v>
+      </c>
+      <c r="B8" s="28" t="n">
+        <f aca="false">(Допущения!$B$30+Допущения!$B$31)*Допущения!$B$5</f>
+        <v>30432.6</v>
+      </c>
+      <c r="C8" s="36" t="n">
+        <f aca="false">IF(Допущения!$B$32=0,0,B8/(12*Допущения!$B$32))</f>
+        <v>0.0488754625346901</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="34" t="s">
+        <v>180</v>
+      </c>
+      <c r="B12" s="37" t="n">
+        <f aca="false">Допущения!$B$34*Допущения!$B$35</f>
+        <v>9500</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="34" t="s">
+        <v>182</v>
+      </c>
+      <c r="B13" s="38" t="n">
+        <f aca="false">'Юнит-экономика'!B30</f>
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1907,95 +2569,95 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>125</v>
+        <v>184</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>126</v>
+        <v>185</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>127</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="B4" s="24" t="s">
-        <v>129</v>
-      </c>
-      <c r="C4" s="24" t="s">
-        <v>130</v>
+      <c r="A4" s="34" t="s">
+        <v>187</v>
+      </c>
+      <c r="B4" s="34" t="s">
+        <v>188</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
-        <v>131</v>
-      </c>
-      <c r="B5" s="24" t="s">
-        <v>132</v>
-      </c>
-      <c r="C5" s="24" t="s">
-        <v>133</v>
+      <c r="A5" s="34" t="s">
+        <v>190</v>
+      </c>
+      <c r="B5" s="34" t="s">
+        <v>191</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
-        <v>134</v>
-      </c>
-      <c r="B6" s="24" t="s">
-        <v>135</v>
-      </c>
-      <c r="C6" s="24" t="s">
-        <v>136</v>
+      <c r="A6" s="34" t="s">
+        <v>193</v>
+      </c>
+      <c r="B6" s="34" t="s">
+        <v>194</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="B7" s="24" t="s">
-        <v>138</v>
-      </c>
-      <c r="C7" s="24" t="s">
-        <v>139</v>
+      <c r="A7" s="34" t="s">
+        <v>196</v>
+      </c>
+      <c r="B7" s="34" t="s">
+        <v>197</v>
+      </c>
+      <c r="C7" s="34" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="24" t="s">
-        <v>140</v>
-      </c>
-      <c r="B8" s="24" t="s">
-        <v>141</v>
-      </c>
-      <c r="C8" s="24" t="s">
-        <v>142</v>
+      <c r="A8" s="34" t="s">
+        <v>199</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>200</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="24" t="s">
-        <v>143</v>
-      </c>
-      <c r="B9" s="24" t="s">
-        <v>144</v>
-      </c>
-      <c r="C9" s="24" t="s">
-        <v>145</v>
+      <c r="A9" s="34" t="s">
+        <v>202</v>
+      </c>
+      <c r="B9" s="34" t="s">
+        <v>203</v>
+      </c>
+      <c r="C9" s="34" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="24" t="s">
-        <v>146</v>
-      </c>
-      <c r="B10" s="24" t="s">
-        <v>147</v>
-      </c>
-      <c r="C10" s="24" t="s">
-        <v>148</v>
+      <c r="A10" s="34" t="s">
+        <v>205</v>
+      </c>
+      <c r="B10" s="34" t="s">
+        <v>206</v>
+      </c>
+      <c r="C10" s="34" t="s">
+        <v>207</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Business: survey answers sheet (Van Westendorp + subscription price ladder) with automatic summary
</commit_message>
<xml_diff>
--- a/business/afib_unit_economics.xlsx
+++ b/business/afib_unit_economics.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Плата и сборка" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Юнит-экономика" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Сравнение" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Чего не хватает" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Опрос — ответы" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Чего не хватает" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="254">
   <si>
     <t xml:space="preserve">AFib Monitor — допущения для цены и юнит-экономики</t>
   </si>
@@ -573,6 +574,144 @@
   </si>
   <si>
     <t xml:space="preserve">Подписчиков для окупаемости сервера (из «Юнит-экономики»)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ответы пациентов (анкета RU/KY). Одна строка — один человек, без имён и телефонов.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пример заполнения (не входит в подсчёт):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">пример</t>
+  </si>
+  <si>
+    <t xml:space="preserve">да</t>
+  </si>
+  <si>
+    <t xml:space="preserve">возможно</t>
+  </si>
+  <si>
+    <t xml:space="preserve">нет</t>
+  </si>
+  <si>
+    <t xml:space="preserve">проверки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">дети</t>
+  </si>
+  <si>
+    <t xml:space="preserve">точность, отчёт врачу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Android</t>
+  </si>
+  <si>
+    <t xml:space="preserve">№</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кто (1 пациент, 2 родств.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Возраст (1: 18–39, 2: 40–59, 3: 60–74, 4: 75+)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ритм по словам врача (да/нет/не знаю)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ЭКГ/Холтер за год, раз</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Последний раз, сом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В5 Слишком дёшево, сом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В6 Выгодно, сом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В7 Дорого, но купил бы, сом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В8 Слишком дорого, сом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В9 Подписка 390 (да/возможно/нет)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В9 250 (да/нет)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В9 590 (да/нет)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В10 Электроды в мес, сом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В11 Ношение (всегда/ночью/проверки/при симптомах)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В12 Кто платит</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В13 Главное (2 пункта)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В14 Телефон (Android/iPhone/кнопочный/нет)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итоги (считаются сами)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Анкет заполнено</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Медиана: слишком дёшево (В5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Медиана: выгодно (В6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Медиана: дорого, но купил бы (В7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Медиана: слишком дорого (В8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Наша цена устройства (из «Допущений»)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доля, кто купил бы по нашей цене (наша цена ≤ В7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доля, для кого наша цена слишком дорогая (≥ В8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Подписка 390: «да»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Подписка 390: «да» или «возможно»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Из сказавших «нет» на 390 — «да» на 250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Из сказавших «да» на 390 — «да» на 590</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Медиана: готовы платить за электроды в месяц</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Себестоимость электродов в месяц (из расчёта)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Хотят носить всегда</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Хотят проверки несколько раз в день</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Метод цен В5–В8 — Van Westendorp (Price Sensitivity Meter). При &lt; 20 анкет выводы предварительные.</t>
   </si>
   <si>
     <t xml:space="preserve">Чего не хватает для полной себестоимости</t>
@@ -786,7 +925,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -940,6 +1079,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2559,6 +2706,1375 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:U55"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>12000</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="N3" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="O3" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="P3" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q3" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="R3" s="7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="39" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" s="39" t="s">
+        <v>194</v>
+      </c>
+      <c r="C5" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="D5" s="39" t="s">
+        <v>196</v>
+      </c>
+      <c r="E5" s="39" t="s">
+        <v>197</v>
+      </c>
+      <c r="F5" s="39" t="s">
+        <v>198</v>
+      </c>
+      <c r="G5" s="39" t="s">
+        <v>199</v>
+      </c>
+      <c r="H5" s="39" t="s">
+        <v>200</v>
+      </c>
+      <c r="I5" s="39" t="s">
+        <v>201</v>
+      </c>
+      <c r="J5" s="39" t="s">
+        <v>202</v>
+      </c>
+      <c r="K5" s="39" t="s">
+        <v>203</v>
+      </c>
+      <c r="L5" s="39" t="s">
+        <v>204</v>
+      </c>
+      <c r="M5" s="39" t="s">
+        <v>205</v>
+      </c>
+      <c r="N5" s="39" t="s">
+        <v>206</v>
+      </c>
+      <c r="O5" s="39" t="s">
+        <v>207</v>
+      </c>
+      <c r="P5" s="39" t="s">
+        <v>208</v>
+      </c>
+      <c r="Q5" s="39" t="s">
+        <v>209</v>
+      </c>
+      <c r="R5" s="39" t="s">
+        <v>210</v>
+      </c>
+      <c r="T5" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="17"/>
+      <c r="N6" s="17"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
+      <c r="T6" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="U6" s="38" t="n">
+        <f aca="false">COUNTA('Опрос — ответы'!$B$6:$B$55)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="17"/>
+      <c r="L7" s="17"/>
+      <c r="M7" s="17"/>
+      <c r="N7" s="17"/>
+      <c r="O7" s="17"/>
+      <c r="P7" s="17"/>
+      <c r="Q7" s="17"/>
+      <c r="R7" s="17"/>
+      <c r="T7" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="U7" s="35" t="n">
+        <f aca="false">IF(COUNT('Опрос — ответы'!$G$6:$G$55)=0,0,MEDIAN('Опрос — ответы'!$G$6:$G$55))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="17"/>
+      <c r="L8" s="17"/>
+      <c r="M8" s="17"/>
+      <c r="N8" s="17"/>
+      <c r="O8" s="17"/>
+      <c r="P8" s="17"/>
+      <c r="Q8" s="17"/>
+      <c r="R8" s="17"/>
+      <c r="T8" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="U8" s="35" t="n">
+        <f aca="false">IF(COUNT('Опрос — ответы'!$H$6:$H$55)=0,0,MEDIAN('Опрос — ответы'!$H$6:$H$55))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="17"/>
+      <c r="M9" s="17"/>
+      <c r="N9" s="17"/>
+      <c r="O9" s="17"/>
+      <c r="P9" s="17"/>
+      <c r="Q9" s="17"/>
+      <c r="R9" s="17"/>
+      <c r="T9" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="U9" s="35" t="n">
+        <f aca="false">IF(COUNT('Опрос — ответы'!$I$6:$I$55)=0,0,MEDIAN('Опрос — ответы'!$I$6:$I$55))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="17"/>
+      <c r="M10" s="17"/>
+      <c r="N10" s="17"/>
+      <c r="O10" s="17"/>
+      <c r="P10" s="17"/>
+      <c r="Q10" s="17"/>
+      <c r="R10" s="17"/>
+      <c r="T10" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="U10" s="35" t="n">
+        <f aca="false">IF(COUNT('Опрос — ответы'!$J$6:$J$55)=0,0,MEDIAN('Опрос — ответы'!$J$6:$J$55))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
+      <c r="L11" s="17"/>
+      <c r="M11" s="17"/>
+      <c r="N11" s="17"/>
+      <c r="O11" s="17"/>
+      <c r="P11" s="17"/>
+      <c r="Q11" s="17"/>
+      <c r="R11" s="17"/>
+      <c r="T11" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="U11" s="35" t="n">
+        <f aca="false">Допущения!$B$22</f>
+        <v>6900</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="17"/>
+      <c r="L12" s="17"/>
+      <c r="M12" s="17"/>
+      <c r="N12" s="17"/>
+      <c r="O12" s="17"/>
+      <c r="P12" s="17"/>
+      <c r="Q12" s="17"/>
+      <c r="R12" s="17"/>
+      <c r="T12" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="U12" s="40" t="n">
+        <f aca="false">IF(COUNT('Опрос — ответы'!$I$6:$I$55)=0,0,COUNTIF('Опрос — ответы'!$I$6:$I$55,"&gt;="&amp;U11)/COUNT('Опрос — ответы'!$I$6:$I$55))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="17"/>
+      <c r="M13" s="17"/>
+      <c r="N13" s="17"/>
+      <c r="O13" s="17"/>
+      <c r="P13" s="17"/>
+      <c r="Q13" s="17"/>
+      <c r="R13" s="17"/>
+      <c r="T13" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="U13" s="40" t="n">
+        <f aca="false">IF(COUNT('Опрос — ответы'!$J$6:$J$55)=0,0,COUNTIF('Опрос — ответы'!$J$6:$J$55,"&lt;="&amp;U11)/COUNT('Опрос — ответы'!$J$6:$J$55))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17"/>
+      <c r="M14" s="17"/>
+      <c r="N14" s="17"/>
+      <c r="O14" s="17"/>
+      <c r="P14" s="17"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="17"/>
+      <c r="T14" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="U14" s="40" t="n">
+        <f aca="false">IF(COUNTA('Опрос — ответы'!$K$6:$K$55)=0,0,COUNTIF('Опрос — ответы'!$K$6:$K$55,"да")/COUNTA('Опрос — ответы'!$K$6:$K$55))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="17"/>
+      <c r="M15" s="17"/>
+      <c r="N15" s="17"/>
+      <c r="O15" s="17"/>
+      <c r="P15" s="17"/>
+      <c r="Q15" s="17"/>
+      <c r="R15" s="17"/>
+      <c r="T15" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="U15" s="40" t="n">
+        <f aca="false">IF(COUNTA('Опрос — ответы'!$K$6:$K$55)=0,0,(COUNTIF('Опрос — ответы'!$K$6:$K$55,"да")+COUNTIF('Опрос — ответы'!$K$6:$K$55,"возможно"))/COUNTA('Опрос — ответы'!$K$6:$K$55))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="17"/>
+      <c r="K16" s="17"/>
+      <c r="L16" s="17"/>
+      <c r="M16" s="17"/>
+      <c r="N16" s="17"/>
+      <c r="O16" s="17"/>
+      <c r="P16" s="17"/>
+      <c r="Q16" s="17"/>
+      <c r="R16" s="17"/>
+      <c r="T16" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="U16" s="40" t="n">
+        <f aca="false">IF(COUNTIF('Опрос — ответы'!$K$6:$K$55,"нет")=0,0,COUNTIF('Опрос — ответы'!$L$6:$L$55,"да")/COUNTIF('Опрос — ответы'!$K$6:$K$55,"нет"))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="17"/>
+      <c r="M17" s="17"/>
+      <c r="N17" s="17"/>
+      <c r="O17" s="17"/>
+      <c r="P17" s="17"/>
+      <c r="Q17" s="17"/>
+      <c r="R17" s="17"/>
+      <c r="T17" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="U17" s="40" t="n">
+        <f aca="false">IF(COUNTIF('Опрос — ответы'!$K$6:$K$55,"да")=0,0,COUNTIF('Опрос — ответы'!$M$6:$M$55,"да")/COUNTIF('Опрос — ответы'!$K$6:$K$55,"да"))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="17"/>
+      <c r="L18" s="17"/>
+      <c r="M18" s="17"/>
+      <c r="N18" s="17"/>
+      <c r="O18" s="17"/>
+      <c r="P18" s="17"/>
+      <c r="Q18" s="17"/>
+      <c r="R18" s="17"/>
+      <c r="T18" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="U18" s="35" t="n">
+        <f aca="false">IF(COUNT('Опрос — ответы'!$N$6:$N$55)=0,0,MEDIAN('Опрос — ответы'!$N$6:$N$55))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="17"/>
+      <c r="L19" s="17"/>
+      <c r="M19" s="17"/>
+      <c r="N19" s="17"/>
+      <c r="O19" s="17"/>
+      <c r="P19" s="17"/>
+      <c r="Q19" s="17"/>
+      <c r="R19" s="17"/>
+      <c r="T19" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="U19" s="35" t="n">
+        <f aca="false">'Юнит-экономика'!B21</f>
+        <v>865.755</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="17"/>
+      <c r="M20" s="17"/>
+      <c r="N20" s="17"/>
+      <c r="O20" s="17"/>
+      <c r="P20" s="17"/>
+      <c r="Q20" s="17"/>
+      <c r="R20" s="17"/>
+      <c r="T20" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="U20" s="40" t="n">
+        <f aca="false">IF(COUNTA('Опрос — ответы'!$O$6:$O$55)=0,0,COUNTIF('Опрос — ответы'!$O$6:$O$55,"всегда")/COUNTA('Опрос — ответы'!$O$6:$O$55))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="17"/>
+      <c r="M21" s="17"/>
+      <c r="N21" s="17"/>
+      <c r="O21" s="17"/>
+      <c r="P21" s="17"/>
+      <c r="Q21" s="17"/>
+      <c r="R21" s="17"/>
+      <c r="T21" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="U21" s="40" t="n">
+        <f aca="false">IF(COUNTA('Опрос — ответы'!$O$6:$O$55)=0,0,COUNTIF('Опрос — ответы'!$O$6:$O$55,"проверки")/COUNTA('Опрос — ответы'!$O$6:$O$55))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="17"/>
+      <c r="K22" s="17"/>
+      <c r="L22" s="17"/>
+      <c r="M22" s="17"/>
+      <c r="N22" s="17"/>
+      <c r="O22" s="17"/>
+      <c r="P22" s="17"/>
+      <c r="Q22" s="17"/>
+      <c r="R22" s="17"/>
+      <c r="T22" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="U22" s="40" t="n">
+        <f aca="false">IF(COUNTA('Опрос — ответы'!$R$6:$R$55)=0,0,COUNTIF('Опрос — ответы'!$R$6:$R$55,"Android")/COUNTA('Опрос — ответы'!$R$6:$R$55))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="17"/>
+      <c r="M23" s="17"/>
+      <c r="N23" s="17"/>
+      <c r="O23" s="17"/>
+      <c r="P23" s="17"/>
+      <c r="Q23" s="17"/>
+      <c r="R23" s="17"/>
+    </row>
+    <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="17"/>
+      <c r="M24" s="17"/>
+      <c r="N24" s="17"/>
+      <c r="O24" s="17"/>
+      <c r="P24" s="17"/>
+      <c r="Q24" s="17"/>
+      <c r="R24" s="17"/>
+      <c r="T24" s="8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="17"/>
+      <c r="M25" s="17"/>
+      <c r="N25" s="17"/>
+      <c r="O25" s="17"/>
+      <c r="P25" s="17"/>
+      <c r="Q25" s="17"/>
+      <c r="R25" s="17"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="17"/>
+      <c r="K26" s="17"/>
+      <c r="L26" s="17"/>
+      <c r="M26" s="17"/>
+      <c r="N26" s="17"/>
+      <c r="O26" s="17"/>
+      <c r="P26" s="17"/>
+      <c r="Q26" s="17"/>
+      <c r="R26" s="17"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="17"/>
+      <c r="L27" s="17"/>
+      <c r="M27" s="17"/>
+      <c r="N27" s="17"/>
+      <c r="O27" s="17"/>
+      <c r="P27" s="17"/>
+      <c r="Q27" s="17"/>
+      <c r="R27" s="17"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="17"/>
+      <c r="L28" s="17"/>
+      <c r="M28" s="17"/>
+      <c r="N28" s="17"/>
+      <c r="O28" s="17"/>
+      <c r="P28" s="17"/>
+      <c r="Q28" s="17"/>
+      <c r="R28" s="17"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="17"/>
+      <c r="L29" s="17"/>
+      <c r="M29" s="17"/>
+      <c r="N29" s="17"/>
+      <c r="O29" s="17"/>
+      <c r="P29" s="17"/>
+      <c r="Q29" s="17"/>
+      <c r="R29" s="17"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="17"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="17"/>
+      <c r="J30" s="17"/>
+      <c r="K30" s="17"/>
+      <c r="L30" s="17"/>
+      <c r="M30" s="17"/>
+      <c r="N30" s="17"/>
+      <c r="O30" s="17"/>
+      <c r="P30" s="17"/>
+      <c r="Q30" s="17"/>
+      <c r="R30" s="17"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="17"/>
+      <c r="H31" s="17"/>
+      <c r="I31" s="17"/>
+      <c r="J31" s="17"/>
+      <c r="K31" s="17"/>
+      <c r="L31" s="17"/>
+      <c r="M31" s="17"/>
+      <c r="N31" s="17"/>
+      <c r="O31" s="17"/>
+      <c r="P31" s="17"/>
+      <c r="Q31" s="17"/>
+      <c r="R31" s="17"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="17"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="17"/>
+      <c r="J32" s="17"/>
+      <c r="K32" s="17"/>
+      <c r="L32" s="17"/>
+      <c r="M32" s="17"/>
+      <c r="N32" s="17"/>
+      <c r="O32" s="17"/>
+      <c r="P32" s="17"/>
+      <c r="Q32" s="17"/>
+      <c r="R32" s="17"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B33" s="17"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
+      <c r="H33" s="17"/>
+      <c r="I33" s="17"/>
+      <c r="J33" s="17"/>
+      <c r="K33" s="17"/>
+      <c r="L33" s="17"/>
+      <c r="M33" s="17"/>
+      <c r="N33" s="17"/>
+      <c r="O33" s="17"/>
+      <c r="P33" s="17"/>
+      <c r="Q33" s="17"/>
+      <c r="R33" s="17"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="17"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="17"/>
+      <c r="J34" s="17"/>
+      <c r="K34" s="17"/>
+      <c r="L34" s="17"/>
+      <c r="M34" s="17"/>
+      <c r="N34" s="17"/>
+      <c r="O34" s="17"/>
+      <c r="P34" s="17"/>
+      <c r="Q34" s="17"/>
+      <c r="R34" s="17"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B35" s="17"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="17"/>
+      <c r="H35" s="17"/>
+      <c r="I35" s="17"/>
+      <c r="J35" s="17"/>
+      <c r="K35" s="17"/>
+      <c r="L35" s="17"/>
+      <c r="M35" s="17"/>
+      <c r="N35" s="17"/>
+      <c r="O35" s="17"/>
+      <c r="P35" s="17"/>
+      <c r="Q35" s="17"/>
+      <c r="R35" s="17"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="17"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="17"/>
+      <c r="J36" s="17"/>
+      <c r="K36" s="17"/>
+      <c r="L36" s="17"/>
+      <c r="M36" s="17"/>
+      <c r="N36" s="17"/>
+      <c r="O36" s="17"/>
+      <c r="P36" s="17"/>
+      <c r="Q36" s="17"/>
+      <c r="R36" s="17"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="17"/>
+      <c r="H37" s="17"/>
+      <c r="I37" s="17"/>
+      <c r="J37" s="17"/>
+      <c r="K37" s="17"/>
+      <c r="L37" s="17"/>
+      <c r="M37" s="17"/>
+      <c r="N37" s="17"/>
+      <c r="O37" s="17"/>
+      <c r="P37" s="17"/>
+      <c r="Q37" s="17"/>
+      <c r="R37" s="17"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="n">
+        <v>33</v>
+      </c>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="17"/>
+      <c r="H38" s="17"/>
+      <c r="I38" s="17"/>
+      <c r="J38" s="17"/>
+      <c r="K38" s="17"/>
+      <c r="L38" s="17"/>
+      <c r="M38" s="17"/>
+      <c r="N38" s="17"/>
+      <c r="O38" s="17"/>
+      <c r="P38" s="17"/>
+      <c r="Q38" s="17"/>
+      <c r="R38" s="17"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" s="17"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="17"/>
+      <c r="G39" s="17"/>
+      <c r="H39" s="17"/>
+      <c r="I39" s="17"/>
+      <c r="J39" s="17"/>
+      <c r="K39" s="17"/>
+      <c r="L39" s="17"/>
+      <c r="M39" s="17"/>
+      <c r="N39" s="17"/>
+      <c r="O39" s="17"/>
+      <c r="P39" s="17"/>
+      <c r="Q39" s="17"/>
+      <c r="R39" s="17"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" s="17"/>
+      <c r="C40" s="17"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="17"/>
+      <c r="F40" s="17"/>
+      <c r="G40" s="17"/>
+      <c r="H40" s="17"/>
+      <c r="I40" s="17"/>
+      <c r="J40" s="17"/>
+      <c r="K40" s="17"/>
+      <c r="L40" s="17"/>
+      <c r="M40" s="17"/>
+      <c r="N40" s="17"/>
+      <c r="O40" s="17"/>
+      <c r="P40" s="17"/>
+      <c r="Q40" s="17"/>
+      <c r="R40" s="17"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" s="17"/>
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="17"/>
+      <c r="G41" s="17"/>
+      <c r="H41" s="17"/>
+      <c r="I41" s="17"/>
+      <c r="J41" s="17"/>
+      <c r="K41" s="17"/>
+      <c r="L41" s="17"/>
+      <c r="M41" s="17"/>
+      <c r="N41" s="17"/>
+      <c r="O41" s="17"/>
+      <c r="P41" s="17"/>
+      <c r="Q41" s="17"/>
+      <c r="R41" s="17"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" s="17"/>
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
+      <c r="E42" s="17"/>
+      <c r="F42" s="17"/>
+      <c r="G42" s="17"/>
+      <c r="H42" s="17"/>
+      <c r="I42" s="17"/>
+      <c r="J42" s="17"/>
+      <c r="K42" s="17"/>
+      <c r="L42" s="17"/>
+      <c r="M42" s="17"/>
+      <c r="N42" s="17"/>
+      <c r="O42" s="17"/>
+      <c r="P42" s="17"/>
+      <c r="Q42" s="17"/>
+      <c r="R42" s="17"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="B43" s="17"/>
+      <c r="C43" s="17"/>
+      <c r="D43" s="17"/>
+      <c r="E43" s="17"/>
+      <c r="F43" s="17"/>
+      <c r="G43" s="17"/>
+      <c r="H43" s="17"/>
+      <c r="I43" s="17"/>
+      <c r="J43" s="17"/>
+      <c r="K43" s="17"/>
+      <c r="L43" s="17"/>
+      <c r="M43" s="17"/>
+      <c r="N43" s="17"/>
+      <c r="O43" s="17"/>
+      <c r="P43" s="17"/>
+      <c r="Q43" s="17"/>
+      <c r="R43" s="17"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="7" t="n">
+        <v>39</v>
+      </c>
+      <c r="B44" s="17"/>
+      <c r="C44" s="17"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="17"/>
+      <c r="F44" s="17"/>
+      <c r="G44" s="17"/>
+      <c r="H44" s="17"/>
+      <c r="I44" s="17"/>
+      <c r="J44" s="17"/>
+      <c r="K44" s="17"/>
+      <c r="L44" s="17"/>
+      <c r="M44" s="17"/>
+      <c r="N44" s="17"/>
+      <c r="O44" s="17"/>
+      <c r="P44" s="17"/>
+      <c r="Q44" s="17"/>
+      <c r="R44" s="17"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" s="17"/>
+      <c r="C45" s="17"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="17"/>
+      <c r="F45" s="17"/>
+      <c r="G45" s="17"/>
+      <c r="H45" s="17"/>
+      <c r="I45" s="17"/>
+      <c r="J45" s="17"/>
+      <c r="K45" s="17"/>
+      <c r="L45" s="17"/>
+      <c r="M45" s="17"/>
+      <c r="N45" s="17"/>
+      <c r="O45" s="17"/>
+      <c r="P45" s="17"/>
+      <c r="Q45" s="17"/>
+      <c r="R45" s="17"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" s="17"/>
+      <c r="C46" s="17"/>
+      <c r="D46" s="17"/>
+      <c r="E46" s="17"/>
+      <c r="F46" s="17"/>
+      <c r="G46" s="17"/>
+      <c r="H46" s="17"/>
+      <c r="I46" s="17"/>
+      <c r="J46" s="17"/>
+      <c r="K46" s="17"/>
+      <c r="L46" s="17"/>
+      <c r="M46" s="17"/>
+      <c r="N46" s="17"/>
+      <c r="O46" s="17"/>
+      <c r="P46" s="17"/>
+      <c r="Q46" s="17"/>
+      <c r="R46" s="17"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" s="17"/>
+      <c r="C47" s="17"/>
+      <c r="D47" s="17"/>
+      <c r="E47" s="17"/>
+      <c r="F47" s="17"/>
+      <c r="G47" s="17"/>
+      <c r="H47" s="17"/>
+      <c r="I47" s="17"/>
+      <c r="J47" s="17"/>
+      <c r="K47" s="17"/>
+      <c r="L47" s="17"/>
+      <c r="M47" s="17"/>
+      <c r="N47" s="17"/>
+      <c r="O47" s="17"/>
+      <c r="P47" s="17"/>
+      <c r="Q47" s="17"/>
+      <c r="R47" s="17"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="7" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" s="17"/>
+      <c r="C48" s="17"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="17"/>
+      <c r="F48" s="17"/>
+      <c r="G48" s="17"/>
+      <c r="H48" s="17"/>
+      <c r="I48" s="17"/>
+      <c r="J48" s="17"/>
+      <c r="K48" s="17"/>
+      <c r="L48" s="17"/>
+      <c r="M48" s="17"/>
+      <c r="N48" s="17"/>
+      <c r="O48" s="17"/>
+      <c r="P48" s="17"/>
+      <c r="Q48" s="17"/>
+      <c r="R48" s="17"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="17"/>
+      <c r="C49" s="17"/>
+      <c r="D49" s="17"/>
+      <c r="E49" s="17"/>
+      <c r="F49" s="17"/>
+      <c r="G49" s="17"/>
+      <c r="H49" s="17"/>
+      <c r="I49" s="17"/>
+      <c r="J49" s="17"/>
+      <c r="K49" s="17"/>
+      <c r="L49" s="17"/>
+      <c r="M49" s="17"/>
+      <c r="N49" s="17"/>
+      <c r="O49" s="17"/>
+      <c r="P49" s="17"/>
+      <c r="Q49" s="17"/>
+      <c r="R49" s="17"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="17"/>
+      <c r="C50" s="17"/>
+      <c r="D50" s="17"/>
+      <c r="E50" s="17"/>
+      <c r="F50" s="17"/>
+      <c r="G50" s="17"/>
+      <c r="H50" s="17"/>
+      <c r="I50" s="17"/>
+      <c r="J50" s="17"/>
+      <c r="K50" s="17"/>
+      <c r="L50" s="17"/>
+      <c r="M50" s="17"/>
+      <c r="N50" s="17"/>
+      <c r="O50" s="17"/>
+      <c r="P50" s="17"/>
+      <c r="Q50" s="17"/>
+      <c r="R50" s="17"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" s="17"/>
+      <c r="C51" s="17"/>
+      <c r="D51" s="17"/>
+      <c r="E51" s="17"/>
+      <c r="F51" s="17"/>
+      <c r="G51" s="17"/>
+      <c r="H51" s="17"/>
+      <c r="I51" s="17"/>
+      <c r="J51" s="17"/>
+      <c r="K51" s="17"/>
+      <c r="L51" s="17"/>
+      <c r="M51" s="17"/>
+      <c r="N51" s="17"/>
+      <c r="O51" s="17"/>
+      <c r="P51" s="17"/>
+      <c r="Q51" s="17"/>
+      <c r="R51" s="17"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="7" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" s="17"/>
+      <c r="C52" s="17"/>
+      <c r="D52" s="17"/>
+      <c r="E52" s="17"/>
+      <c r="F52" s="17"/>
+      <c r="G52" s="17"/>
+      <c r="H52" s="17"/>
+      <c r="I52" s="17"/>
+      <c r="J52" s="17"/>
+      <c r="K52" s="17"/>
+      <c r="L52" s="17"/>
+      <c r="M52" s="17"/>
+      <c r="N52" s="17"/>
+      <c r="O52" s="17"/>
+      <c r="P52" s="17"/>
+      <c r="Q52" s="17"/>
+      <c r="R52" s="17"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="7" t="n">
+        <v>48</v>
+      </c>
+      <c r="B53" s="17"/>
+      <c r="C53" s="17"/>
+      <c r="D53" s="17"/>
+      <c r="E53" s="17"/>
+      <c r="F53" s="17"/>
+      <c r="G53" s="17"/>
+      <c r="H53" s="17"/>
+      <c r="I53" s="17"/>
+      <c r="J53" s="17"/>
+      <c r="K53" s="17"/>
+      <c r="L53" s="17"/>
+      <c r="M53" s="17"/>
+      <c r="N53" s="17"/>
+      <c r="O53" s="17"/>
+      <c r="P53" s="17"/>
+      <c r="Q53" s="17"/>
+      <c r="R53" s="17"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7" t="n">
+        <v>49</v>
+      </c>
+      <c r="B54" s="17"/>
+      <c r="C54" s="17"/>
+      <c r="D54" s="17"/>
+      <c r="E54" s="17"/>
+      <c r="F54" s="17"/>
+      <c r="G54" s="17"/>
+      <c r="H54" s="17"/>
+      <c r="I54" s="17"/>
+      <c r="J54" s="17"/>
+      <c r="K54" s="17"/>
+      <c r="L54" s="17"/>
+      <c r="M54" s="17"/>
+      <c r="N54" s="17"/>
+      <c r="O54" s="17"/>
+      <c r="P54" s="17"/>
+      <c r="Q54" s="17"/>
+      <c r="R54" s="17"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="B55" s="17"/>
+      <c r="C55" s="17"/>
+      <c r="D55" s="17"/>
+      <c r="E55" s="17"/>
+      <c r="F55" s="17"/>
+      <c r="G55" s="17"/>
+      <c r="H55" s="17"/>
+      <c r="I55" s="17"/>
+      <c r="J55" s="17"/>
+      <c r="K55" s="17"/>
+      <c r="L55" s="17"/>
+      <c r="M55" s="17"/>
+      <c r="N55" s="17"/>
+      <c r="O55" s="17"/>
+      <c r="P55" s="17"/>
+      <c r="Q55" s="17"/>
+      <c r="R55" s="17"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2569,95 +4085,95 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>183</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>184</v>
+        <v>230</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>185</v>
+        <v>231</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>186</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="34" t="s">
-        <v>187</v>
+        <v>233</v>
       </c>
       <c r="B4" s="34" t="s">
-        <v>188</v>
+        <v>234</v>
       </c>
       <c r="C4" s="34" t="s">
-        <v>189</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="34" t="s">
-        <v>190</v>
+        <v>236</v>
       </c>
       <c r="B5" s="34" t="s">
-        <v>191</v>
+        <v>237</v>
       </c>
       <c r="C5" s="34" t="s">
-        <v>192</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="34" t="s">
-        <v>193</v>
+        <v>239</v>
       </c>
       <c r="B6" s="34" t="s">
-        <v>194</v>
+        <v>240</v>
       </c>
       <c r="C6" s="34" t="s">
-        <v>195</v>
+        <v>241</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="34" t="s">
-        <v>196</v>
+        <v>242</v>
       </c>
       <c r="B7" s="34" t="s">
-        <v>197</v>
+        <v>243</v>
       </c>
       <c r="C7" s="34" t="s">
-        <v>198</v>
+        <v>244</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="34" t="s">
-        <v>199</v>
+        <v>245</v>
       </c>
       <c r="B8" s="34" t="s">
-        <v>200</v>
+        <v>246</v>
       </c>
       <c r="C8" s="34" t="s">
-        <v>201</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="34" t="s">
-        <v>202</v>
+        <v>248</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>203</v>
+        <v>249</v>
       </c>
       <c r="C9" s="34" t="s">
-        <v>204</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="34" t="s">
-        <v>205</v>
+        <v>251</v>
       </c>
       <c r="B10" s="34" t="s">
-        <v>206</v>
+        <v>252</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>207</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Business: electrodes gap updated with Notebook 15
</commit_message>
<xml_diff>
--- a/business/afib_unit_economics.xlsx
+++ b/business/afib_unit_economics.xlsx
@@ -765,10 +765,10 @@
     <t xml:space="preserve">Сколько электродов реально уходит в месяц</t>
   </si>
   <si>
-    <t xml:space="preserve">Главный расход; допущение 45 шт — не измерено</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Стенд + 5–10 пациентов</t>
+    <t xml:space="preserve">Главный расход; допущение 45 шт — не измерено. Ноутбук 15 (ml/WEAR_MODES.md): для поиска редкой ФП нужно постоянное ношение; для контроля частой ФП хватит 2–3 проверок в день с многоразовыми электродами — тогда расходников нет</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Стенд + 5–10 пациентов; версия с многоразовыми электродами — разработка</t>
   </si>
   <si>
     <t xml:space="preserve">Цена электродов у местных поставщиков (Бишкек, Гуанчжоу)</t>

</xml_diff>

<commit_message>
Hardware: patch v1 schematic as code (AD8232 front end from SparkFun reference, ESP32-S3-MINI-1, USB-C, MCP73831, ME6211), netlist, JLCPCB BOM, rules check OK; workbook part counts from the schematic
</commit_message>
<xml_diff>
--- a/business/afib_unit_economics.xlsx
+++ b/business/afib_unit_economics.xlsx
@@ -246,7 +246,7 @@
     <t xml:space="preserve">Плата и сборка: детали (LCSC) и сборка (JLCPCB, Economic PCBA)</t>
   </si>
   <si>
-    <t xml:space="preserve">Цены деталей — за 1 шт при ~100 шт (если нет тарифа 100+ — ближайший). Пайки — по числу выводов корпуса, ОЦЕНКА: проверить по футпринтам. Главные детали (ESP32, AD8232, аккумулятор) — на листе «Допущения».</t>
+    <t xml:space="preserve">Цены деталей — за 1 шт при ~100 шт (если нет тарифа 100+ — ближайший). Пайки — по числу выводов корпуса. Светодиод и кнопка пока не посчитаны. Главные детали (ESP32, AD8232, аккумулятор) — на листе «Допущения».</t>
   </si>
   <si>
     <t xml:space="preserve">Деталь</t>
@@ -312,22 +312,22 @@
     <t xml:space="preserve">lcsc.com/product-detail/C131337.html, 20+: $0.0358; паяется вручную</t>
   </si>
   <si>
-    <t xml:space="preserve">Резисторы 0402 (обвязка AD8232, делитель батареи, светодиод)</t>
+    <t xml:space="preserve">Резисторы 0402 (все 22 по схеме hardware/patch_v1)</t>
   </si>
   <si>
     <t xml:space="preserve">C25744</t>
   </si>
   <si>
-    <t xml:space="preserve">lcsc.com/product-detail/C25744.html, 100+: $0.0016. Количество — ОЦЕНКА по типовой схеме AD8232</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Конденсаторы 0402 100 нФ и др.</t>
+    <t xml:space="preserve">Количество — по схеме (design.py). Цена — как у 10 кОм C25744 ($0.0016, 100+); номиналы 10 МОм, 1,4 МОм и др. ещё не выбраны на LCSC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Конденсаторы (все 15 по схеме)</t>
   </si>
   <si>
     <t xml:space="preserve">C1525</t>
   </si>
   <si>
-    <t xml:space="preserve">lcsc.com/product-detail/C1525.html, 100+: $0.004. Количество — ОЦЕНКА</t>
+    <t xml:space="preserve">Количество — по схеме. Цена — как у 100 нФ C1525 ($0.004); 22 мкФ и 4,7 мкФ дороже — уточнить</t>
   </si>
   <si>
     <t xml:space="preserve">ESP32-S3-MINI-1 и AD8232 (пайки; цены — на листе «Допущения»)</t>
@@ -1450,7 +1450,7 @@
       </c>
       <c r="B10" s="10" t="n">
         <f aca="false">'Плата и сборка'!$B$31</f>
-        <v>1.855</v>
+        <v>1.9102</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>12</v>
@@ -1963,7 +1963,7 @@
         <v>96</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="D9" s="18" t="n">
         <v>0.0016</v>
@@ -1973,13 +1973,13 @@
       </c>
       <c r="F9" s="19" t="n">
         <f aca="false">C9*D9</f>
-        <v>0.0192</v>
+        <v>0.0352</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
         <v>98</v>
       </c>
@@ -1987,7 +1987,7 @@
         <v>99</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D10" s="18" t="n">
         <v>0.004</v>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="F10" s="19" t="n">
         <f aca="false">C10*D10</f>
-        <v>0.056</v>
+        <v>0.06</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>100</v>
@@ -2122,7 +2122,7 @@
       </c>
       <c r="B23" s="23" t="n">
         <f aca="false">SUM(F4:F10)</f>
-        <v>0.8283</v>
+        <v>0.8483</v>
       </c>
       <c r="G23" s="7"/>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="B24" s="24" t="n">
         <f aca="false">SUMPRODUCT(C4:C11,E4:E11)-C8*E8</f>
-        <v>173</v>
+        <v>195</v>
       </c>
       <c r="G24" s="7" t="s">
         <v>122</v>
@@ -2144,7 +2144,7 @@
       </c>
       <c r="B25" s="23" t="n">
         <f aca="false">B24*B16</f>
-        <v>0.2768</v>
+        <v>0.312</v>
       </c>
       <c r="G25" s="7"/>
     </row>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="B31" s="26" t="n">
         <f aca="false">B23+B25+B26+B27+B29</f>
-        <v>1.855</v>
+        <v>1.9102</v>
       </c>
       <c r="G31" s="7" t="s">
         <v>130</v>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="B4" s="27" t="n">
         <f aca="false">Допущения!$B$7+Допущения!$B$8+Допущения!$B$9+Допущения!$B$10</f>
-        <v>16.8278</v>
+        <v>16.883</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>134</v>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="B5" s="28" t="n">
         <f aca="false">B4*Допущения!$B$5</f>
-        <v>1471.59111</v>
+        <v>1476.41835</v>
       </c>
       <c r="E5" s="7"/>
     </row>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="B7" s="28" t="n">
         <f aca="false">B6-B5</f>
-        <v>5428.40889</v>
+        <v>5423.58165</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>137</v>
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B8" s="29" t="n">
         <f aca="false">IF(B6=0,0,B7/B6)</f>
-        <v>0.786725926086957</v>
+        <v>0.786026326086957</v>
       </c>
       <c r="E8" s="7"/>
     </row>

</xml_diff>

<commit_message>
Hardware: all 26 BOM lines with LCSC numbers checked on lcsc.com (board parts $10.18), KiCad netlist with footprints (Espressif ESP32-S3-MINI-1 footprint included), pins checked against footprint pads in CI; workbook small parts from the BOM (device without enclosure $17.20)
</commit_message>
<xml_diff>
--- a/business/afib_unit_economics.xlsx
+++ b/business/afib_unit_economics.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="305">
   <si>
     <t xml:space="preserve">AFib Monitor — допущения для цены и юнит-экономики</t>
   </si>
@@ -246,7 +246,7 @@
     <t xml:space="preserve">Плата и сборка: детали (LCSC) и сборка (JLCPCB, Economic PCBA)</t>
   </si>
   <si>
-    <t xml:space="preserve">Цены деталей — за 1 шт при ~100 шт (если нет тарифа 100+ — ближайший). Пайки — по числу выводов корпуса. Светодиод и кнопка пока не посчитаны. Главные детали (ESP32, AD8232, аккумулятор) — на листе «Допущения».</t>
+    <t xml:space="preserve">Все детали платы из BOM схемы (hardware/patch_v1), цены LCSC за 1 шт при ~100 шт (если нет тарифа 100+ — ближайший). Пайки — по числу выводов корпуса. Главные детали (ESP32, AD8232, аккумулятор) — на листе «Допущения».</t>
   </si>
   <si>
     <t xml:space="preserve">Деталь</t>
@@ -267,67 +267,220 @@
     <t xml:space="preserve">Сумма, $</t>
   </si>
   <si>
-    <t xml:space="preserve">Зарядка LiPo MCP73831T-2ACI/OT</t>
+    <t xml:space="preserve">1.5nF (C1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C23967</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C23967.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.7uF (C11,C12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C19666</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C19666.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1nF (C2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1523</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C1523.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10nF (C3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C15195</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C15195.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.33uF (C4,C6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C159798</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C159798.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1uF (C5,C7,C10,C15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1525</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C1525.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1uF (C8,C13,C14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C52923</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C52923.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22uF (C9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C45783</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C45783.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED charging (D1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2286</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C2286.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.5 mm jack, electrode cable (J1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5123133</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C5123133.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB-C receptacle 16P (J2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C165948</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C165948.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battery connector JST PH 2P (J3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C131337</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C131337.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10M (R1,R2,R10,R11,R13,R14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C26086</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C26086.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.4M (R12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C270644</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C270644.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10k (R15,R16,R19)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C25744</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C25744.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.1k (R17,R18)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C25905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C25905.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1k (R20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C11702</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C11702.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">180k (R3,R4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C25760</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C25760.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">360k (R5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C45956</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C45956.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1M (R6,R7,R9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C26083</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C26083.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100k (R8,R21,R22)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C25741</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C25741.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOOT button (SW1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C49234124</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lcsc.com/product-detail/C49234124.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCP73831T-2ACI/OT (U3)</t>
   </si>
   <si>
     <t xml:space="preserve">C424093</t>
   </si>
   <si>
-    <t xml:space="preserve">lcsc.com/product-detail/C424093.html, 100+: $0.4483</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Стабилизатор 3.3 В ME6211C33M5G-N</t>
+    <t xml:space="preserve">lcsc.com/product-detail/C424093.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME6211C33M5G-N (U4)</t>
   </si>
   <si>
     <t xml:space="preserve">C82942</t>
   </si>
   <si>
-    <t xml:space="preserve">lcsc.com/product-detail/C82942.html, 100+: $0.0503</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Разъём USB-C TYPE-C-31-M-12 (16 конт.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C165948</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lcsc.com/product-detail/C165948.html, 50+: $0.1368 (тарифа 100+ нет)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Гнездо 3.5 мм для кабеля электродов KH-PJ-321A-SMT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5123133</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lcsc.com/product-detail/C5123133.html, 50+: $0.0819 (большая из двух цен)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Разъём аккумулятора JST B2B-PH-K-S (выводной)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C131337</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lcsc.com/product-detail/C131337.html, 20+: $0.0358; паяется вручную</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Резисторы 0402 (все 22 по схеме hardware/patch_v1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C25744</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Количество — по схеме (design.py). Цена — как у 10 кОм C25744 ($0.0016, 100+); номиналы 10 МОм, 1,4 МОм и др. ещё не выбраны на LCSC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Конденсаторы (все 15 по схеме)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1525</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Количество — по схеме. Цена — как у 100 нФ C1525 ($0.004); 22 мкФ и 4,7 мкФ дороже — уточнить</t>
+    <t xml:space="preserve">lcsc.com/product-detail/C82942.html, проверено 20.10.2026; список — hardware/patch_v1/bom_jlcpcb.csv</t>
   </si>
   <si>
     <t xml:space="preserve">ESP32-S3-MINI-1 и AD8232 (пайки; цены — на листе «Допущения»)</t>
@@ -729,7 +882,7 @@
     <t xml:space="preserve">Корпус и кабель к электродам; точная цена платы для 100 шт</t>
   </si>
   <si>
-    <t xml:space="preserve">Плата и сборка посчитаны по тарифам, но корпус не посчитан; цена самой платы взята как акция $2 за 5 шт</t>
+    <t xml:space="preserve">Детали платы посчитаны по BOM с номерами LCSC, сборка — по тарифам; корпус не посчитан; цена самой платы — акция $2 за 5 шт</t>
   </si>
   <si>
     <t xml:space="preserve">Я: схема в KiCad → калькулятор JLCPCB; корпус — 3D-печать или литьё</t>
@@ -1449,8 +1602,8 @@
         <v>18</v>
       </c>
       <c r="B10" s="10" t="n">
-        <f aca="false">'Плата и сборка'!$B$31</f>
-        <v>1.9102</v>
+        <f aca="false">'Плата и сборка'!$B$48</f>
+        <v>2.2235</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>12</v>
@@ -1784,7 +1937,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -1835,7 +1988,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
         <v>80</v>
       </c>
@@ -1846,20 +1999,20 @@
         <v>1</v>
       </c>
       <c r="D4" s="18" t="n">
-        <v>0.4483</v>
+        <v>0.0092</v>
       </c>
       <c r="E4" s="17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F4" s="19" t="n">
         <f aca="false">C4*D4</f>
-        <v>0.4483</v>
+        <v>0.0092</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
         <v>83</v>
       </c>
@@ -1867,23 +2020,23 @@
         <v>84</v>
       </c>
       <c r="C5" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>0.0503</v>
+        <v>0.0163</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F5" s="19" t="n">
         <f aca="false">C5*D5</f>
-        <v>0.0503</v>
+        <v>0.0326</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
         <v>86</v>
       </c>
@@ -1894,20 +2047,20 @@
         <v>1</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>0.1368</v>
+        <v>0.0039</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="F6" s="19" t="n">
         <f aca="false">C6*D6</f>
-        <v>0.1368</v>
+        <v>0.0039</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
         <v>89</v>
       </c>
@@ -1918,20 +2071,20 @@
         <v>1</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>0.0819</v>
+        <v>0.0041</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F7" s="19" t="n">
         <f aca="false">C7*D7</f>
-        <v>0.0819</v>
+        <v>0.0041</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
         <v>92</v>
       </c>
@@ -1939,17 +2092,17 @@
         <v>93</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="18" t="n">
-        <v>0.0358</v>
+        <v>0.0208</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>2</v>
       </c>
       <c r="F8" s="19" t="n">
         <f aca="false">C8*D8</f>
-        <v>0.0358</v>
+        <v>0.0416</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>94</v>
@@ -1963,17 +2116,17 @@
         <v>96</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="D9" s="18" t="n">
-        <v>0.0016</v>
+        <v>0.004</v>
       </c>
       <c r="E9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="F9" s="19" t="n">
         <f aca="false">C9*D9</f>
-        <v>0.0352</v>
+        <v>0.016</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>97</v>
@@ -1987,219 +2140,627 @@
         <v>99</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D10" s="18" t="n">
-        <v>0.004</v>
+        <v>0.0068</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>2</v>
       </c>
       <c r="F10" s="19" t="n">
         <f aca="false">C10*D10</f>
-        <v>0.06</v>
+        <v>0.0204</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
         <v>101</v>
       </c>
-      <c r="C11" s="0" t="n">
+      <c r="B11" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="D11" s="18" t="n">
+        <v>0.1959</v>
+      </c>
       <c r="E11" s="17" t="n">
-        <v>86</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <f aca="false">C11*D11</f>
+        <v>0.1959</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <f aca="false">C12*D12</f>
+        <v>0.0077</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>103</v>
-      </c>
-      <c r="B13" s="20" t="n">
+        <v>107</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="18" t="n">
+        <v>0.0819</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <f aca="false">C13*D13</f>
+        <v>0.0819</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>0.1368</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <f aca="false">C14*D14</f>
+        <v>0.1368</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>0.0358</v>
+      </c>
+      <c r="E15" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="7" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>105</v>
-      </c>
-      <c r="B14" s="21" t="n">
-        <v>100</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>107</v>
-      </c>
-      <c r="B15" s="21" t="n">
+      <c r="F15" s="19" t="n">
+        <f aca="false">C15*D15</f>
+        <v>0.0358</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="C16" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="G15" s="7" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>109</v>
-      </c>
-      <c r="B16" s="18" t="n">
+      <c r="D16" s="18" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="19" t="n">
+        <f aca="false">C16*D16</f>
+        <v>0.0168</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="19" t="n">
+        <f aca="false">C17*D17</f>
+        <v>0.0008</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="C18" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="18" t="n">
         <v>0.0016</v>
       </c>
-      <c r="G16" s="7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
-        <v>111</v>
-      </c>
-      <c r="B17" s="18" t="n">
-        <v>0.0164</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
-        <v>113</v>
-      </c>
-      <c r="B18" s="22" t="n">
-        <v>8.18</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E18" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <f aca="false">C18*D18</f>
+        <v>0.0048</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>115</v>
-      </c>
-      <c r="B19" s="22" t="n">
-        <v>1.53</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>125</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="C19" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="18" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="E19" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="19" t="n">
+        <f aca="false">C19*D19</f>
+        <v>0.0046</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="B20" s="22" t="n">
-        <v>3.07</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>128</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="18" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="E20" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="19" t="n">
+        <f aca="false">C20*D20</f>
+        <v>0.0013</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="B21" s="22" t="n">
-        <v>3.58</v>
-      </c>
-      <c r="G21" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>131</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="C21" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="18" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="E21" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="19" t="n">
+        <f aca="false">C21*D21</f>
+        <v>0.0034</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="C22" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="18" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="E22" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="19" t="n">
+        <f aca="false">C22*D22</f>
+        <v>0.0019</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>120</v>
-      </c>
-      <c r="B23" s="23" t="n">
-        <f aca="false">SUM(F4:F10)</f>
-        <v>0.8483</v>
-      </c>
-      <c r="G23" s="7"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>137</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="C23" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" s="18" t="n">
+        <v>0.0024</v>
+      </c>
+      <c r="E23" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" s="19" t="n">
+        <f aca="false">C23*D23</f>
+        <v>0.0072</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>121</v>
-      </c>
-      <c r="B24" s="24" t="n">
-        <f aca="false">SUMPRODUCT(C4:C11,E4:E11)-C8*E8</f>
-        <v>195</v>
-      </c>
-      <c r="G24" s="7" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>140</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="C24" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" s="18" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" s="19" t="n">
+        <f aca="false">C24*D24</f>
+        <v>0.0045</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>123</v>
-      </c>
-      <c r="B25" s="23" t="n">
-        <f aca="false">B24*B16</f>
-        <v>0.312</v>
-      </c>
-      <c r="G25" s="7"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>143</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="C25" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="18" t="n">
+        <v>0.0254</v>
+      </c>
+      <c r="E25" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="19" t="n">
+        <f aca="false">C25*D25</f>
+        <v>0.0254</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>124</v>
-      </c>
-      <c r="B26" s="23" t="n">
-        <f aca="false">C8*E8*B17</f>
-        <v>0.0328</v>
-      </c>
-      <c r="G26" s="7"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>146</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="18" t="n">
+        <v>0.4483</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F26" s="19" t="n">
+        <f aca="false">C26*D26</f>
+        <v>0.4483</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="B27" s="23" t="n">
-        <f aca="false">B13/5</f>
-        <v>0.4</v>
-      </c>
-      <c r="G27" s="7"/>
+        <v>149</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="C27" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="18" t="n">
+        <v>0.0503</v>
+      </c>
+      <c r="E27" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F27" s="19" t="n">
+        <f aca="false">C27*D27</f>
+        <v>0.0503</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>126</v>
-      </c>
-      <c r="B28" s="25" t="n">
-        <f aca="false">B18+B19+B15*B20+B21</f>
+        <v>152</v>
+      </c>
+      <c r="C28" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="B30" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="s">
+        <v>156</v>
+      </c>
+      <c r="B31" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="B32" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="G32" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="B33" s="18" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="B34" s="18" t="n">
+        <v>0.0164</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="B35" s="22" t="n">
+        <v>8.18</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="B36" s="22" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="0" t="s">
+        <v>167</v>
+      </c>
+      <c r="B37" s="22" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="B38" s="22" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="B40" s="23" t="n">
+        <f aca="false">SUM(F4:F27)</f>
+        <v>1.1552</v>
+      </c>
+      <c r="G40" s="7"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="B41" s="24" t="n">
+        <f aca="false">SUMPRODUCT(C4:C28,E4:E28)-C15*E15</f>
+        <v>199</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="B42" s="23" t="n">
+        <f aca="false">B41*B33</f>
+        <v>0.3184</v>
+      </c>
+      <c r="G42" s="7"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="B43" s="23" t="n">
+        <f aca="false">C15*E15*B34</f>
+        <v>0.0328</v>
+      </c>
+      <c r="G43" s="7"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="B44" s="23" t="n">
+        <f aca="false">B30/5</f>
+        <v>0.4</v>
+      </c>
+      <c r="G44" s="7"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="0" t="s">
+        <v>177</v>
+      </c>
+      <c r="B45" s="25" t="n">
+        <f aca="false">B35+B36+B32*B37+B38</f>
         <v>31.71</v>
       </c>
-      <c r="G28" s="7" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
-        <v>128</v>
-      </c>
-      <c r="B29" s="23" t="n">
-        <f aca="false">IF(B14=0,0,B28/B14)</f>
+      <c r="G45" s="7" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="0" t="s">
+        <v>179</v>
+      </c>
+      <c r="B46" s="23" t="n">
+        <f aca="false">IF(B31=0,0,B45/B31)</f>
         <v>0.3171</v>
       </c>
-      <c r="G29" s="7"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="B31" s="26" t="n">
-        <f aca="false">B23+B25+B26+B27+B29</f>
-        <v>1.9102</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>130</v>
+      <c r="G46" s="7"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B48" s="26" t="n">
+        <f aca="false">B40+B42+B43+B44+B46</f>
+        <v>2.2235</v>
+      </c>
+      <c r="G48" s="7" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -2231,33 +2792,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>131</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>132</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>133</v>
+        <v>184</v>
       </c>
       <c r="B4" s="27" t="n">
         <f aca="false">Допущения!$B$7+Допущения!$B$8+Допущения!$B$9+Допущения!$B$10</f>
-        <v>16.883</v>
+        <v>17.1963</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>134</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>135</v>
+        <v>186</v>
       </c>
       <c r="B5" s="28" t="n">
         <f aca="false">B4*Допущения!$B$5</f>
-        <v>1476.41835</v>
+        <v>1503.816435</v>
       </c>
       <c r="E5" s="7"/>
     </row>
@@ -2273,34 +2834,34 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>136</v>
+        <v>187</v>
       </c>
       <c r="B7" s="28" t="n">
         <f aca="false">B6-B5</f>
-        <v>5423.58165</v>
+        <v>5396.183565</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>137</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>138</v>
+        <v>189</v>
       </c>
       <c r="B8" s="29" t="n">
         <f aca="false">IF(B6=0,0,B7/B6)</f>
-        <v>0.786026326086957</v>
+        <v>0.782055589130435</v>
       </c>
       <c r="E8" s="7"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>139</v>
+        <v>190</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>140</v>
+        <v>191</v>
       </c>
       <c r="B11" s="11" t="n">
         <v>50</v>
@@ -2312,12 +2873,12 @@
         <v>1000</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>141</v>
+        <v>192</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>142</v>
+        <v>193</v>
       </c>
       <c r="B12" s="28" t="n">
         <f aca="false">Допущения!$B$23</f>
@@ -2335,7 +2896,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>143</v>
+        <v>194</v>
       </c>
       <c r="B13" s="28" t="n">
         <f aca="false">Допущения!$B$23*Допущения!$B$19*Допущения!$B$20</f>
@@ -2353,7 +2914,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B14" s="28" t="n">
         <f aca="false">(Допущения!$B$15+Допущения!$B$16)*Допущения!$B$5/B11</f>
@@ -2368,12 +2929,12 @@
         <v>1.13685</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>145</v>
+        <v>196</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>146</v>
+        <v>197</v>
       </c>
       <c r="B15" s="28" t="n">
         <f aca="false">(Допущения!$B$17/12)*Допущения!$B$5/B11</f>
@@ -2388,12 +2949,12 @@
         <v>0.7214625</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>147</v>
+        <v>198</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>148</v>
+        <v>199</v>
       </c>
       <c r="B16" s="30" t="n">
         <f aca="false">B12-B13-B14-B15</f>
@@ -2408,12 +2969,12 @@
         <v>329.6416875</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>149</v>
+        <v>200</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>150</v>
+        <v>201</v>
       </c>
       <c r="B17" s="28" t="n">
         <f aca="false">B16*B11</f>
@@ -2431,7 +2992,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>151</v>
+        <v>202</v>
       </c>
       <c r="B18" s="30" t="n">
         <f aca="false">B17*12</f>
@@ -2449,36 +3010,36 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>152</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>153</v>
+        <v>204</v>
       </c>
       <c r="B21" s="28" t="n">
         <f aca="false">Допущения!$B$12*Допущения!$B$13*Допущения!$B$5</f>
         <v>865.755</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>154</v>
+        <v>205</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>155</v>
+        <v>206</v>
       </c>
       <c r="B22" s="28" t="n">
         <f aca="false">B21*(1+Допущения!$B$24)</f>
         <v>1038.906</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>156</v>
+        <v>207</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>157</v>
+        <v>208</v>
       </c>
       <c r="B23" s="31" t="n">
         <f aca="false">IF(Допущения!$B$23=0,0,B21/Допущения!$B$23)</f>
@@ -2488,7 +3049,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>158</v>
+        <v>209</v>
       </c>
       <c r="B24" s="28" t="n">
         <f aca="false">Допущения!$B$23+B22</f>
@@ -2498,7 +3059,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>159</v>
+        <v>210</v>
       </c>
       <c r="B25" s="29" t="n">
         <f aca="false">IF(Допущения!$B$32=0,0,B24/Допущения!$B$32)</f>
@@ -2508,12 +3069,12 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>160</v>
+        <v>211</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>161</v>
+        <v>212</v>
       </c>
       <c r="B28" s="32" t="n">
         <f aca="false">(Допущения!$B$15+Допущения!$B$16+Допущения!$B$17/12)*Допущения!$B$5</f>
@@ -2522,7 +3083,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>162</v>
+        <v>213</v>
       </c>
       <c r="B29" s="32" t="n">
         <f aca="false">Допущения!$B$23*(1-Допущения!$B$19*Допущения!$B$20)</f>
@@ -2531,14 +3092,14 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>163</v>
+        <v>214</v>
       </c>
       <c r="B30" s="33" t="n">
         <f aca="false">IF(B29&lt;=0,0,ROUNDUP(B28/B29,0))</f>
         <v>6</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>164</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -2567,26 +3128,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>165</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>166</v>
+        <v>217</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>167</v>
+        <v>218</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>168</v>
+        <v>219</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>169</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="34" t="s">
-        <v>170</v>
+        <v>221</v>
       </c>
       <c r="B4" s="35" t="n">
         <f aca="false">Допущения!$B$22+12*'Юнит-экономика'!B24</f>
@@ -2597,12 +3158,12 @@
         <v>0.0386198350292939</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>171</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="34" t="s">
-        <v>172</v>
+        <v>223</v>
       </c>
       <c r="B5" s="28" t="n">
         <f aca="false">Допущения!$B$22+12*Допущения!$B$23</f>
@@ -2613,12 +3174,12 @@
         <v>0.0185977489978415</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>173</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="34" t="s">
-        <v>174</v>
+        <v>225</v>
       </c>
       <c r="B6" s="28" t="n">
         <f aca="false">4*Допущения!$B$26</f>
@@ -2629,12 +3190,12 @@
         <v>0.00963613937711995</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>175</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="34" t="s">
-        <v>176</v>
+        <v>227</v>
       </c>
       <c r="B7" s="28" t="n">
         <f aca="false">4*Допущения!$B$27</f>
@@ -2645,12 +3206,12 @@
         <v>0.0115633672525439</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>175</v>
+        <v>226</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="34" t="s">
-        <v>177</v>
+        <v>228</v>
       </c>
       <c r="B8" s="28" t="n">
         <f aca="false">(Допущения!$B$30+Допущения!$B$31)*Допущения!$B$5</f>
@@ -2661,29 +3222,29 @@
         <v>0.0488754625346901</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>178</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>179</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="34" t="s">
-        <v>180</v>
+        <v>231</v>
       </c>
       <c r="B12" s="37" t="n">
         <f aca="false">Допущения!$B$34*Допущения!$B$35</f>
         <v>9500</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>181</v>
+        <v>232</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="34" t="s">
-        <v>182</v>
+        <v>233</v>
       </c>
       <c r="B13" s="38" t="n">
         <f aca="false">'Юнит-экономика'!B30</f>
@@ -2716,17 +3277,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>183</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>184</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>1</v>
@@ -2735,7 +3296,7 @@
         <v>3</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>186</v>
+        <v>237</v>
       </c>
       <c r="E3" s="7" t="n">
         <v>2</v>
@@ -2756,85 +3317,85 @@
         <v>12000</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>187</v>
+        <v>238</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7" t="s">
-        <v>188</v>
+        <v>239</v>
       </c>
       <c r="N3" s="7" t="n">
         <v>300</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>189</v>
+        <v>240</v>
       </c>
       <c r="P3" s="7" t="s">
-        <v>190</v>
+        <v>241</v>
       </c>
       <c r="Q3" s="7" t="s">
-        <v>191</v>
+        <v>242</v>
       </c>
       <c r="R3" s="7" t="s">
-        <v>192</v>
+        <v>243</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="39" t="s">
-        <v>193</v>
+        <v>244</v>
       </c>
       <c r="B5" s="39" t="s">
-        <v>194</v>
+        <v>245</v>
       </c>
       <c r="C5" s="39" t="s">
-        <v>195</v>
+        <v>246</v>
       </c>
       <c r="D5" s="39" t="s">
-        <v>196</v>
+        <v>247</v>
       </c>
       <c r="E5" s="39" t="s">
-        <v>197</v>
+        <v>248</v>
       </c>
       <c r="F5" s="39" t="s">
-        <v>198</v>
+        <v>249</v>
       </c>
       <c r="G5" s="39" t="s">
-        <v>199</v>
+        <v>250</v>
       </c>
       <c r="H5" s="39" t="s">
-        <v>200</v>
+        <v>251</v>
       </c>
       <c r="I5" s="39" t="s">
-        <v>201</v>
+        <v>252</v>
       </c>
       <c r="J5" s="39" t="s">
-        <v>202</v>
+        <v>253</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>203</v>
+        <v>254</v>
       </c>
       <c r="L5" s="39" t="s">
-        <v>204</v>
+        <v>255</v>
       </c>
       <c r="M5" s="39" t="s">
-        <v>205</v>
+        <v>256</v>
       </c>
       <c r="N5" s="39" t="s">
-        <v>206</v>
+        <v>257</v>
       </c>
       <c r="O5" s="39" t="s">
-        <v>207</v>
+        <v>258</v>
       </c>
       <c r="P5" s="39" t="s">
-        <v>208</v>
+        <v>259</v>
       </c>
       <c r="Q5" s="39" t="s">
-        <v>209</v>
+        <v>260</v>
       </c>
       <c r="R5" s="39" t="s">
-        <v>210</v>
+        <v>261</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>211</v>
+        <v>262</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2859,7 +3420,7 @@
       <c r="Q6" s="17"/>
       <c r="R6" s="17"/>
       <c r="T6" s="5" t="s">
-        <v>212</v>
+        <v>263</v>
       </c>
       <c r="U6" s="38" t="n">
         <f aca="false">COUNTA('Опрос — ответы'!$B$6:$B$55)</f>
@@ -2888,7 +3449,7 @@
       <c r="Q7" s="17"/>
       <c r="R7" s="17"/>
       <c r="T7" s="5" t="s">
-        <v>213</v>
+        <v>264</v>
       </c>
       <c r="U7" s="35" t="n">
         <f aca="false">IF(COUNT('Опрос — ответы'!$G$6:$G$55)=0,0,MEDIAN('Опрос — ответы'!$G$6:$G$55))</f>
@@ -2917,7 +3478,7 @@
       <c r="Q8" s="17"/>
       <c r="R8" s="17"/>
       <c r="T8" s="5" t="s">
-        <v>214</v>
+        <v>265</v>
       </c>
       <c r="U8" s="35" t="n">
         <f aca="false">IF(COUNT('Опрос — ответы'!$H$6:$H$55)=0,0,MEDIAN('Опрос — ответы'!$H$6:$H$55))</f>
@@ -2946,7 +3507,7 @@
       <c r="Q9" s="17"/>
       <c r="R9" s="17"/>
       <c r="T9" s="5" t="s">
-        <v>215</v>
+        <v>266</v>
       </c>
       <c r="U9" s="35" t="n">
         <f aca="false">IF(COUNT('Опрос — ответы'!$I$6:$I$55)=0,0,MEDIAN('Опрос — ответы'!$I$6:$I$55))</f>
@@ -2975,7 +3536,7 @@
       <c r="Q10" s="17"/>
       <c r="R10" s="17"/>
       <c r="T10" s="5" t="s">
-        <v>216</v>
+        <v>267</v>
       </c>
       <c r="U10" s="35" t="n">
         <f aca="false">IF(COUNT('Опрос — ответы'!$J$6:$J$55)=0,0,MEDIAN('Опрос — ответы'!$J$6:$J$55))</f>
@@ -3004,7 +3565,7 @@
       <c r="Q11" s="17"/>
       <c r="R11" s="17"/>
       <c r="T11" s="5" t="s">
-        <v>217</v>
+        <v>268</v>
       </c>
       <c r="U11" s="35" t="n">
         <f aca="false">Допущения!$B$22</f>
@@ -3033,7 +3594,7 @@
       <c r="Q12" s="17"/>
       <c r="R12" s="17"/>
       <c r="T12" s="5" t="s">
-        <v>218</v>
+        <v>269</v>
       </c>
       <c r="U12" s="40" t="n">
         <f aca="false">IF(COUNT('Опрос — ответы'!$I$6:$I$55)=0,0,COUNTIF('Опрос — ответы'!$I$6:$I$55,"&gt;="&amp;U11)/COUNT('Опрос — ответы'!$I$6:$I$55))</f>
@@ -3062,7 +3623,7 @@
       <c r="Q13" s="17"/>
       <c r="R13" s="17"/>
       <c r="T13" s="5" t="s">
-        <v>219</v>
+        <v>270</v>
       </c>
       <c r="U13" s="40" t="n">
         <f aca="false">IF(COUNT('Опрос — ответы'!$J$6:$J$55)=0,0,COUNTIF('Опрос — ответы'!$J$6:$J$55,"&lt;="&amp;U11)/COUNT('Опрос — ответы'!$J$6:$J$55))</f>
@@ -3091,7 +3652,7 @@
       <c r="Q14" s="17"/>
       <c r="R14" s="17"/>
       <c r="T14" s="5" t="s">
-        <v>220</v>
+        <v>271</v>
       </c>
       <c r="U14" s="40" t="n">
         <f aca="false">IF(COUNTA('Опрос — ответы'!$K$6:$K$55)=0,0,COUNTIF('Опрос — ответы'!$K$6:$K$55,"да")/COUNTA('Опрос — ответы'!$K$6:$K$55))</f>
@@ -3120,7 +3681,7 @@
       <c r="Q15" s="17"/>
       <c r="R15" s="17"/>
       <c r="T15" s="5" t="s">
-        <v>221</v>
+        <v>272</v>
       </c>
       <c r="U15" s="40" t="n">
         <f aca="false">IF(COUNTA('Опрос — ответы'!$K$6:$K$55)=0,0,(COUNTIF('Опрос — ответы'!$K$6:$K$55,"да")+COUNTIF('Опрос — ответы'!$K$6:$K$55,"возможно"))/COUNTA('Опрос — ответы'!$K$6:$K$55))</f>
@@ -3149,7 +3710,7 @@
       <c r="Q16" s="17"/>
       <c r="R16" s="17"/>
       <c r="T16" s="5" t="s">
-        <v>222</v>
+        <v>273</v>
       </c>
       <c r="U16" s="40" t="n">
         <f aca="false">IF(COUNTIF('Опрос — ответы'!$K$6:$K$55,"нет")=0,0,COUNTIF('Опрос — ответы'!$L$6:$L$55,"да")/COUNTIF('Опрос — ответы'!$K$6:$K$55,"нет"))</f>
@@ -3178,7 +3739,7 @@
       <c r="Q17" s="17"/>
       <c r="R17" s="17"/>
       <c r="T17" s="5" t="s">
-        <v>223</v>
+        <v>274</v>
       </c>
       <c r="U17" s="40" t="n">
         <f aca="false">IF(COUNTIF('Опрос — ответы'!$K$6:$K$55,"да")=0,0,COUNTIF('Опрос — ответы'!$M$6:$M$55,"да")/COUNTIF('Опрос — ответы'!$K$6:$K$55,"да"))</f>
@@ -3207,7 +3768,7 @@
       <c r="Q18" s="17"/>
       <c r="R18" s="17"/>
       <c r="T18" s="5" t="s">
-        <v>224</v>
+        <v>275</v>
       </c>
       <c r="U18" s="35" t="n">
         <f aca="false">IF(COUNT('Опрос — ответы'!$N$6:$N$55)=0,0,MEDIAN('Опрос — ответы'!$N$6:$N$55))</f>
@@ -3236,7 +3797,7 @@
       <c r="Q19" s="17"/>
       <c r="R19" s="17"/>
       <c r="T19" s="5" t="s">
-        <v>225</v>
+        <v>276</v>
       </c>
       <c r="U19" s="35" t="n">
         <f aca="false">'Юнит-экономика'!B21</f>
@@ -3265,7 +3826,7 @@
       <c r="Q20" s="17"/>
       <c r="R20" s="17"/>
       <c r="T20" s="5" t="s">
-        <v>226</v>
+        <v>277</v>
       </c>
       <c r="U20" s="40" t="n">
         <f aca="false">IF(COUNTA('Опрос — ответы'!$O$6:$O$55)=0,0,COUNTIF('Опрос — ответы'!$O$6:$O$55,"всегда")/COUNTA('Опрос — ответы'!$O$6:$O$55))</f>
@@ -3294,7 +3855,7 @@
       <c r="Q21" s="17"/>
       <c r="R21" s="17"/>
       <c r="T21" s="5" t="s">
-        <v>227</v>
+        <v>278</v>
       </c>
       <c r="U21" s="40" t="n">
         <f aca="false">IF(COUNTA('Опрос — ответы'!$O$6:$O$55)=0,0,COUNTIF('Опрос — ответы'!$O$6:$O$55,"проверки")/COUNTA('Опрос — ответы'!$O$6:$O$55))</f>
@@ -3323,7 +3884,7 @@
       <c r="Q22" s="17"/>
       <c r="R22" s="17"/>
       <c r="T22" s="5" t="s">
-        <v>192</v>
+        <v>243</v>
       </c>
       <c r="U22" s="40" t="n">
         <f aca="false">IF(COUNTA('Опрос — ответы'!$R$6:$R$55)=0,0,COUNTIF('Опрос — ответы'!$R$6:$R$55,"Android")/COUNTA('Опрос — ответы'!$R$6:$R$55))</f>
@@ -3374,7 +3935,7 @@
       <c r="Q24" s="17"/>
       <c r="R24" s="17"/>
       <c r="T24" s="8" t="s">
-        <v>228</v>
+        <v>279</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4085,95 +4646,95 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>229</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>230</v>
+        <v>281</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>231</v>
+        <v>282</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>232</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="34" t="s">
-        <v>233</v>
+        <v>284</v>
       </c>
       <c r="B4" s="34" t="s">
-        <v>234</v>
+        <v>285</v>
       </c>
       <c r="C4" s="34" t="s">
-        <v>235</v>
+        <v>286</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="34" t="s">
-        <v>236</v>
+        <v>287</v>
       </c>
       <c r="B5" s="34" t="s">
-        <v>237</v>
+        <v>288</v>
       </c>
       <c r="C5" s="34" t="s">
-        <v>238</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="34" t="s">
-        <v>239</v>
+        <v>290</v>
       </c>
       <c r="B6" s="34" t="s">
-        <v>240</v>
+        <v>291</v>
       </c>
       <c r="C6" s="34" t="s">
-        <v>241</v>
+        <v>292</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="34" t="s">
-        <v>242</v>
+        <v>293</v>
       </c>
       <c r="B7" s="34" t="s">
-        <v>243</v>
+        <v>294</v>
       </c>
       <c r="C7" s="34" t="s">
-        <v>244</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="34" t="s">
-        <v>245</v>
+        <v>296</v>
       </c>
       <c r="B8" s="34" t="s">
-        <v>246</v>
+        <v>297</v>
       </c>
       <c r="C8" s="34" t="s">
-        <v>247</v>
+        <v>298</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="34" t="s">
-        <v>248</v>
+        <v>299</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>249</v>
+        <v>300</v>
       </c>
       <c r="C9" s="34" t="s">
-        <v>250</v>
+        <v>301</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="34" t="s">
-        <v>251</v>
+        <v>302</v>
       </c>
       <c r="B10" s="34" t="s">
-        <v>252</v>
+        <v>303</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>253</v>
+        <v>304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>